<commit_message>
edit award number (no effect on XML)
</commit_message>
<xml_diff>
--- a/nes-lter-doc-transect-info.xlsx
+++ b/nes-lter-doc-transect-info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmorkeski\Documents\nes-lter-doc-transect\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4190C2C-E652-4F40-98E3-718E24FD9205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55F060FD-59DB-4C4C-9A4A-D165F9A5C7C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ColumnHeaders" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="131">
   <si>
     <t>micromolePerLiter</t>
   </si>
@@ -408,21 +408,6 @@
   </si>
   <si>
     <t>OCE-2322676</t>
-  </si>
-  <si>
-    <t>OCE-2322677</t>
-  </si>
-  <si>
-    <t>OCE-2322678</t>
-  </si>
-  <si>
-    <t>OCE-2322679</t>
-  </si>
-  <si>
-    <t>OCE-2322680</t>
-  </si>
-  <si>
-    <t>OCE-2322681</t>
   </si>
   <si>
     <t>Date of laboratory sample analysis (Kujawinski lab) or date data received (Carlson lab)</t>
@@ -1208,7 +1193,7 @@
         <v>93</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>77</v>
@@ -1642,7 +1627,7 @@
         <v>28</v>
       </c>
       <c r="J3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1666,15 +1651,15 @@
         <v>28</v>
       </c>
       <c r="J4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B5" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C5" t="s">
         <v>33</v>
@@ -1698,7 +1683,7 @@
         <v>28</v>
       </c>
       <c r="J5" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1727,7 +1712,7 @@
         <v>28</v>
       </c>
       <c r="J6" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1756,25 +1741,25 @@
         <v>28</v>
       </c>
       <c r="J7" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="C8" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="D8" t="s">
         <v>24</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="F8"/>
       <c r="G8" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="H8" t="s">
         <v>24</v>

</xml_diff>